<commit_message>
feat: implement full-stack schedule management and class member enrollment features
</commit_message>
<xml_diff>
--- a/Owly_UseCases.xlsx
+++ b/Owly_UseCases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Owly\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data\Owly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70782336-245C-4557-BD60-108A3DAC951A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F4E709-52A5-4F01-8B52-C70E3BE876A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3345" yWindow="2070" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EMS SaaS Plan" sheetId="1" r:id="rId1"/>
@@ -1626,282 +1626,282 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" s="3" t="s">
+      <c r="C19" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="3" t="s">
+      <c r="C20" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="3" t="s">
+      <c r="C21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D22" s="3" t="s">
+      <c r="C22" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="3" t="s">
+      <c r="C23" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="3" t="s">
+      <c r="C24" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D25" s="3" t="s">
+      <c r="C25" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="C26" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" s="3" t="s">
+      <c r="C27" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D28" s="3" t="s">
+      <c r="C28" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" s="3" t="s">
+      <c r="C29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D30" s="3" t="s">
+      <c r="C30" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D31" s="3" t="s">
+      <c r="C31" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="3" t="s">
+      <c r="C32" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="7" t="s">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement authentication management with token refreshing and session persistence features.
</commit_message>
<xml_diff>
--- a/Owly_UseCases.xlsx
+++ b/Owly_UseCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data\Owly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F4E709-52A5-4F01-8B52-C70E3BE876A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE57BF3D-DDBB-4BED-ABF5-C310E19DA523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1262,7 +1262,7 @@
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="75" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="6" max="6" width="40.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1906,122 +1906,122 @@
       </c>
     </row>
     <row r="33" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" s="3" t="s">
+      <c r="C33" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D34" s="3" t="s">
+      <c r="C34" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" s="3" t="s">
+      <c r="C35" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D36" s="3" t="s">
+      <c r="C36" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D37" s="3" t="s">
+      <c r="C37" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D38" s="3" t="s">
+      <c r="C38" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="7" t="s">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement grade category management service and dashboard UI components
</commit_message>
<xml_diff>
--- a/Owly_UseCases.xlsx
+++ b/Owly_UseCases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Owly\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data\Owly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417AD2FE-2597-432F-9C93-FDE064F136ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EAAC6EE-5698-4FF0-89DF-B1DED29D79B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EMS SaaS Plan" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="279">
   <si>
     <t>ID</t>
   </si>
@@ -851,13 +851,19 @@
   </si>
   <si>
     <t>Tệp ảnh chụp biên lai chuyển khoản thành công gửi lên cho Giáo viên đối soát duyệt (Pending).</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Chưa làm student</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -881,6 +887,12 @@
       <color rgb="FF111111"/>
       <name val="Segoe UI"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -902,7 +914,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -925,11 +937,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE0E0E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE0E0E0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -951,6 +974,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1254,7 +1280,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr defaultRowHeight="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1263,9 +1289,10 @@
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="75" customWidth="1"/>
     <col min="6" max="6" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1284,8 +1311,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -1305,7 +1335,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
@@ -1325,7 +1355,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -1345,7 +1375,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
@@ -1365,7 +1395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1385,7 +1415,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>25</v>
       </c>
@@ -1405,7 +1435,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>29</v>
       </c>
@@ -1425,7 +1455,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>32</v>
       </c>
@@ -1445,7 +1475,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
@@ -1465,7 +1495,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
@@ -1485,7 +1515,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
@@ -1505,7 +1535,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>48</v>
       </c>
@@ -1525,7 +1555,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>52</v>
       </c>
@@ -1545,7 +1575,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>55</v>
       </c>
@@ -1565,7 +1595,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>59</v>
       </c>
@@ -1905,7 +1935,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>117</v>
       </c>
@@ -1925,7 +1955,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>121</v>
       </c>
@@ -1945,7 +1975,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>124</v>
       </c>
@@ -1965,7 +1995,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>127</v>
       </c>
@@ -1985,7 +2015,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>130</v>
       </c>
@@ -2005,7 +2035,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>134</v>
       </c>
@@ -2025,7 +2055,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>137</v>
       </c>
@@ -2045,47 +2075,53 @@
         <v>141</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
+    <row r="40" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="7" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
+      <c r="G40" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="F41" s="7" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G41" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>149</v>
       </c>
@@ -2105,7 +2141,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>152</v>
       </c>
@@ -2125,187 +2161,196 @@
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+    <row r="44" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D44" s="3" t="s">
+      <c r="C44" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="F44" s="7" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+    <row r="45" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D45" s="3" t="s">
+      <c r="C45" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="F45" s="4" t="s">
+      <c r="F45" s="7" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
+    <row r="46" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="F46" s="7" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
+      <c r="G46" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C47" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="F47" s="4" t="s">
+      <c r="F47" s="7" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
+      <c r="G47" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D48" s="3" t="s">
+      <c r="C48" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F48" s="7" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
+    <row r="49" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B49" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D49" s="3" t="s">
+      <c r="C49" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="E49" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="F49" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
+    <row r="50" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E50" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="F50" s="7" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
+      <c r="G50" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D51" s="3" t="s">
+      <c r="C51" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="E51" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="F51" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
+    <row r="52" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D52" s="3" t="s">
+      <c r="C52" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D52" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="E52" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="F52" s="4" t="s">
+      <c r="F52" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>185</v>
       </c>
@@ -2325,7 +2370,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>188</v>
       </c>
@@ -2345,7 +2390,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>191</v>
       </c>
@@ -2365,7 +2410,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>194</v>
       </c>
@@ -2385,7 +2430,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>197</v>
       </c>
@@ -2405,7 +2450,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>200</v>
       </c>
@@ -2425,47 +2470,47 @@
         <v>175</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="2" t="s">
+    <row r="59" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D59" s="3" t="s">
+      <c r="C59" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="E59" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="F59" s="4" t="s">
+      <c r="F59" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
+    <row r="60" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="B60" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D60" s="3" t="s">
+      <c r="C60" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D60" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="E60" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="F60" s="4" t="s">
+      <c r="F60" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>210</v>
       </c>
@@ -2485,7 +2530,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>213</v>
       </c>
@@ -2505,7 +2550,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>216</v>
       </c>
@@ -2525,7 +2570,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>219</v>
       </c>
@@ -2867,6 +2912,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement student class scheduling and management features with session tracking and attendance support
</commit_message>
<xml_diff>
--- a/Owly_UseCases.xlsx
+++ b/Owly_UseCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data\Owly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EAAC6EE-5698-4FF0-89DF-B1DED29D79B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC652EF4-C1D5-43D2-A334-249ABD2C3842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2511,22 +2511,22 @@
       </c>
     </row>
     <row r="61" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D61" s="3" t="s">
+      <c r="C61" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D61" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="E61" s="3" t="s">
+      <c r="E61" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="F61" s="4" t="s">
+      <c r="F61" s="7" t="s">
         <v>175</v>
       </c>
     </row>
@@ -2671,42 +2671,42 @@
       </c>
     </row>
     <row r="69" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="2" t="s">
+      <c r="A69" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="B69" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="C69" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D69" s="3" t="s">
+      <c r="C69" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D69" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="E69" s="3" t="s">
+      <c r="E69" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="F69" s="4" t="s">
+      <c r="F69" s="7" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="2" t="s">
+      <c r="A70" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B70" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D70" s="3" t="s">
+      <c r="C70" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D70" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E70" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="F70" s="4" t="s">
+      <c r="F70" s="7" t="s">
         <v>226</v>
       </c>
     </row>

</xml_diff>